<commit_message>
Add public-safe replication inputs and exports.
Skip the default raw rebuild that depends on restricted product data, publish the prepared analysis datasets needed for reruns, and include the updated manuscript and CT.gov export changes.
</commit_message>
<xml_diff>
--- a/output/tables/manuscript/s6_table_effects_by_food_group.xlsx
+++ b/output/tables/manuscript/s6_table_effects_by_food_group.xlsx
@@ -69,7 +69,7 @@
     <t>1.9</t>
   </si>
   <si>
-    <t>(-0.0, 3.8)</t>
+    <t>(-0.03, 3.8)</t>
   </si>
   <si>
     <t>5.2</t>
@@ -168,10 +168,10 @@
     <t>-0.4</t>
   </si>
   <si>
-    <t>(-0.8, 0.0)</t>
-  </si>
-  <si>
-    <t>0.0</t>
+    <t>(-0.8, 0.04)</t>
+  </si>
+  <si>
+    <t>0.03</t>
   </si>
   <si>
     <t>(-0.4, 0.5)</t>
@@ -222,7 +222,7 @@
     <t>(-1.7, -0.2)</t>
   </si>
   <si>
-    <t>(-1.4, 0.0)</t>
+    <t>(-1.4, 0.05)</t>
   </si>
   <si>
     <t>-2.7</t>
@@ -231,7 +231,7 @@
     <t>(-4.3, -1.0)</t>
   </si>
   <si>
-    <t>-0.0</t>
+    <t>-0.01</t>
   </si>
   <si>
     <t>(-1.6, 1.6)</t>

</xml_diff>